<commit_message>
Update weekly ranking [2026-06-17]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -41,6 +41,7 @@
     <sheet name="magapoke_2026-05-27" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="magapoke_2026-06-03" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11090,6 +11091,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ハプスブルク家の華麗なる受難</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-06-24]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -42,6 +42,7 @@
     <sheet name="magapoke_2026-06-03" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11367,6 +11368,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ダンジョンの測量士～地図で無双するダンジョン攻略～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>おれは美少女VTuber</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-01]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -43,6 +43,7 @@
     <sheet name="magapoke_2026-06-10" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11644,6 +11645,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>アイ・ヘイ・チュー</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>異世界グルメで成り上がり無双～山に追放されたので、のんびりキャンプを楽しんでいたらいつの間にか強くなっていて、王侯貴族や実力者たちが俺を放っておいてくれません。一方、俺を追放した貴族たちは破滅が始まる～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>君が監督！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ダンジョンの測量士～地図で無双するダンジョン攻略～</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-08]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -44,6 +44,7 @@
     <sheet name="magapoke_2026-06-17" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -11921,6 +11922,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>【爆アド】生まれた直後から最強悪霊と脳内バトルしてたら魔力量が測定可能域を超えてました〜悪憑の子の謙虚な覇道〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>顔憑</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-15]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -45,6 +45,7 @@
     <sheet name="magapoke_2026-06-24" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12198,6 +12199,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet39.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>アイドラトリィ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>白鳥運子は31画</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ダンジョンの測量士～地図で無双するダンジョン攻略～</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-22]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -46,6 +46,7 @@
     <sheet name="magapoke_2026-07-01" sheetId="37" state="visible" r:id="rId37"/>
     <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -12941,6 +12942,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet40.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>顔憑</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>皇女転生　～伝説の大魔導士（♂）、姫騎士となりて伝説の令嬢騎士団を作り無双する～</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-07-29]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -47,6 +47,7 @@
     <sheet name="magapoke_2026-07-08" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13218,6 +13219,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>黄昏町プリズナーズ</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>花子狩り</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>顔憑</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ペンの夢に紅をさす</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-05]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -48,6 +48,7 @@
     <sheet name="magapoke_2026-07-15" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13495,6 +13496,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>顔憑</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>俺聖女　～俺が聖女でお前が悪役令嬢　最強タッグで乙女ゲーム完全攻略いたしますわ～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>八田未蘭と青春に上等！！</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>おれは美少女VTuber</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ラブソング</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-12]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -49,6 +49,7 @@
     <sheet name="magapoke_2026-07-22" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet name="magapoke_2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -13772,6 +13773,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>御贖事処 煮るばあな</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>元カノカフェ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ダンジョンの測量士～地図で無双するダンジョン攻略～</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>堕天使ちゃんはがんばれない</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-19]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -50,6 +50,7 @@
     <sheet name="magapoke_2026-07-29" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="magapoke_2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="magapoke_2026-08-19" sheetId="44" state="visible" r:id="rId44"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14049,6 +14050,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet44.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>元カノカフェ</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>御贖事処 煮るばあな</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-08-26]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -51,6 +51,7 @@
     <sheet name="magapoke_2026-08-05" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="magapoke_2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="magapoke_2026-08-19" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="magapoke_2026-08-26" sheetId="45" state="visible" r:id="rId45"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14326,6 +14327,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet45.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>元カノカフェ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>御贖事処 煮るばあな</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-09-02]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -52,6 +52,7 @@
     <sheet name="magapoke_2026-08-12" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="magapoke_2026-08-19" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="magapoke_2026-08-26" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet name="magapoke_2026-09-02" sheetId="46" state="visible" r:id="rId46"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14603,6 +14604,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet46.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>八田未蘭と青春に上等！！</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ラブソング</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>麗しババアは孫が欲しい！</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>元カノカフェ</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>顔憑</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-09-09]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -53,6 +53,7 @@
     <sheet name="magapoke_2026-08-19" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="magapoke_2026-08-26" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="magapoke_2026-09-02" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet name="magapoke_2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14880,6 +14881,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet47.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>元カノカフェ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>御贖事処 煮るばあな</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>八田未蘭と青春に上等！！</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-09-16]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -54,6 +54,7 @@
     <sheet name="magapoke_2026-08-26" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="magapoke_2026-09-02" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="magapoke_2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="magapoke_2026-09-16" sheetId="48" state="visible" r:id="rId48"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15157,6 +15158,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>撮ってはいけない家</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>弱くて可愛い君が好き</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ラブソング</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-09-23]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -55,6 +55,7 @@
     <sheet name="magapoke_2026-09-02" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="magapoke_2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="magapoke_2026-09-16" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="magapoke_2026-09-23" sheetId="49" state="visible" r:id="rId49"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15434,6 +15435,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>撮ってはいけない家</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>弱くて可愛い君が好き</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-09-30]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -56,6 +56,7 @@
     <sheet name="magapoke_2026-09-09" sheetId="47" state="visible" r:id="rId47"/>
     <sheet name="magapoke_2026-09-16" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="magapoke_2026-09-23" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="magapoke_2026-09-30" sheetId="50" state="visible" r:id="rId50"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16167,6 +16168,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>撮ってはいけない家</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>弱くて可愛い君が好き</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-10-07]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -57,6 +57,7 @@
     <sheet name="magapoke_2026-09-16" sheetId="48" state="visible" r:id="rId48"/>
     <sheet name="magapoke_2026-09-23" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="magapoke_2026-09-30" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="magapoke_2026-10-07" sheetId="51" state="visible" r:id="rId51"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16444,6 +16445,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>アイ・ヘイ・チュー</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>解除師カンナの魔術録</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>撮ってはいけない家</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>死に戻り聖女は毒家族と決別する〜未来を変えたら、狂暴王子様の溺愛が待ってました!?〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>極悪令嬢は仁義を貫く</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-10-14]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -58,6 +58,7 @@
     <sheet name="magapoke_2026-09-23" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="magapoke_2026-09-30" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="magapoke_2026-10-07" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="magapoke_2026-10-14" sheetId="52" state="visible" r:id="rId52"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16721,6 +16722,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>裏東京のオソロシドコロ</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>撮ってはいけない家</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ダンジョンの測量士～地図で無双するダンジョン攻略～</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ゲーム開始前に死ぬモブ悪役皇子に転生した俺　～推しヒロインの妹と幸せになるために最弱魔法【闇刃】を過剰な努力で極め抜いたら、最強のぶっ壊れ性能と化していた件～</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ぎるてぃらいぶらり</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>元カノカフェ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-10-21]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -59,6 +59,7 @@
     <sheet name="magapoke_2026-09-30" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="magapoke_2026-10-07" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="magapoke_2026-10-14" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="magapoke_2026-10-21" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16998,6 +16999,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－アグリーダック－</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>まじイヌ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>撮ってはいけない家</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>お母さん冒険者、ログインボーナスでスキル【主婦】に目覚めました。週一貰えるチラシで冒険者生活頑張ります！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>その青春</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>弱くて可愛い君が好き</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>宇宙人と出会う前に読む本</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update weekly ranking [2026-10-28]
</commit_message>
<xml_diff>
--- a/weekly_ranking.xlsx
+++ b/weekly_ranking.xlsx
@@ -60,6 +60,7 @@
     <sheet name="magapoke_2026-10-07" sheetId="51" state="visible" r:id="rId51"/>
     <sheet name="magapoke_2026-10-14" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="magapoke_2026-10-21" sheetId="53" state="visible" r:id="rId53"/>
+    <sheet name="magapoke_2026-10-28" sheetId="54" state="visible" r:id="rId54"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17275,6 +17276,282 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet54.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>36キューピット</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>『無刀』のおっさん、実はラスダン攻略済み</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>排水溝につまったスライムを日々かたづけるだけの底辺職、なぜか実力者たちの熱い視線を集めてしまう</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>あの島の海音荘</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>りりむホリック</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ギークラウン</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>キラーシッター</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ゼロとヒャク</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ズレた解釈のぼくら</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ゲームが進むにつれてどんどん役目がなくなっていく脳筋キャラに転生した俺は、それでも物理を極めることにした</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>怨霊日和</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ヒトの心が読める彼女の話</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>殺し屋の営業術</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>千仙戦記</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>群雄を綴る</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>お前がヤったんだろ！</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>普通の本はありません！</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ジャンクシュート</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ハンドレッドノート－コフィンロビン－</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>クラス転移で拠点魔法を手に入れたら、ハーレム共同生活が始まりました　～絶海の孤島でサバイバルが始まったけど、俺だけが女子と一緒に楽しく快適に生活できるらしい～</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>そして刹那は繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>新宿解消録テンチョウ　みいちゃんと山田さん外伝</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>一億年修行の無自覚剣聖〜ただの棒だと馬鹿にされた万能の神器と、極限の修行で生み出した『剣鬼』の人格で異世界を圧倒する〜</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>弱くて可愛い君が好き</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>闇覚醒して主人公にボコされるかませ犬に憑依したが原作と違いすぎて戸惑ってる</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>